<commit_message>
LISBOA - 26/09/2026 (Paper evaluation: constraint checklist judged with the request date, updated analysis and notebook)
</commit_message>
<xml_diff>
--- a/eval/results/statistics/extended_tables_ablation_final_20260926_141018.xlsx
+++ b/eval/results/statistics/extended_tables_ablation_final_20260926_141018.xlsx
@@ -79636,7 +79636,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>55/58 (0.948); 0; 0</t>
+          <t>55/58 (0.948); 1; 0</t>
         </is>
       </c>
     </row>
@@ -79653,7 +79653,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>53/58 (0.914); 1; 0</t>
+          <t>54/58 (0.931); 3; 0</t>
         </is>
       </c>
     </row>
@@ -79670,7 +79670,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>55/58 (0.948); 3; 0</t>
+          <t>57/58 (0.983); 1; 0</t>
         </is>
       </c>
     </row>
@@ -79687,7 +79687,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>0.914 to 0.966</t>
+          <t>0.948 to 0.966</t>
         </is>
       </c>
     </row>
@@ -79704,7 +79704,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>97.8%, 0.772</t>
+          <t>97.4%, 0.613</t>
         </is>
       </c>
     </row>

</xml_diff>